<commit_message>
installed a new streamlit version
</commit_message>
<xml_diff>
--- a/data/reference_events.xlsx
+++ b/data/reference_events.xlsx
@@ -8,19 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORK\IPC-HQ\RAAP - RISK ANALYSIS APPROACH\AFGHANISTAN\CLIMATOLOGICAL\pythonProject\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{556E7855-BBAF-44E6-95AA-2F4C1350968B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFC4B0C3-E4A4-42E4-A946-DD92490D5AA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="26537" windowHeight="15943" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="4395" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="reference_events" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">reference_events!$A$1:$F$67</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="137">
   <si>
     <t>country</t>
   </si>
@@ -425,6 +428,12 @@
   </si>
   <si>
     <t>Sudan civil war</t>
+  </si>
+  <si>
+    <t>2025-05</t>
+  </si>
+  <si>
+    <t>2025-09</t>
   </si>
 </sst>
 </file>
@@ -789,7 +798,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F67"/>
+  <dimension ref="A1:F68"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="11.23046875" bestFit="1" customWidth="1"/>
@@ -2139,6 +2148,26 @@
         <v>15</v>
       </c>
     </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A68" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="D68" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E68" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F68" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
South Sudan Added and many other changes including indicators added
</commit_message>
<xml_diff>
--- a/data/reference_events.xlsx
+++ b/data/reference_events.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORK\IPC-HQ\RAAP - RISK ANALYSIS APPROACH\AFGHANISTAN\CLIMATOLOGICAL\pythonProject\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFC4B0C3-E4A4-42E4-A946-DD92490D5AA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D22F69A0-B326-4CF7-B9A5-03472F00483A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="4395" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="reference_events" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,20 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">reference_events!$A$1:$F$67</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -799,16 +812,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F68"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.23046875" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="7.4609375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.42578125" customWidth="1"/>
+    <col min="3" max="3" width="7.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="34" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.15234375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.3828125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -828,7 +842,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
@@ -848,7 +862,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -868,7 +882,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -888,7 +902,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
@@ -908,7 +922,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
@@ -928,7 +942,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
@@ -948,7 +962,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>29</v>
       </c>
@@ -968,7 +982,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>29</v>
       </c>
@@ -988,7 +1002,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>29</v>
       </c>
@@ -1008,7 +1022,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>29</v>
       </c>
@@ -1028,7 +1042,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>29</v>
       </c>
@@ -1048,7 +1062,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>29</v>
       </c>
@@ -1068,7 +1082,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>29</v>
       </c>
@@ -1088,7 +1102,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>29</v>
       </c>
@@ -1108,7 +1122,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>29</v>
       </c>
@@ -1128,7 +1142,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>29</v>
       </c>
@@ -1148,7 +1162,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>29</v>
       </c>
@@ -1168,7 +1182,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>29</v>
       </c>
@@ -1188,7 +1202,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>29</v>
       </c>
@@ -1208,7 +1222,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>29</v>
       </c>
@@ -1228,7 +1242,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>29</v>
       </c>
@@ -1248,7 +1262,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>68</v>
       </c>
@@ -1268,7 +1282,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>68</v>
       </c>
@@ -1288,7 +1302,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>68</v>
       </c>
@@ -1308,7 +1322,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>68</v>
       </c>
@@ -1328,7 +1342,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>68</v>
       </c>
@@ -1348,7 +1362,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>68</v>
       </c>
@@ -1368,7 +1382,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>68</v>
       </c>
@@ -1388,7 +1402,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>68</v>
       </c>
@@ -1408,7 +1422,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>68</v>
       </c>
@@ -1428,7 +1442,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>68</v>
       </c>
@@ -1448,7 +1462,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>68</v>
       </c>
@@ -1468,7 +1482,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>68</v>
       </c>
@@ -1488,7 +1502,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>90</v>
       </c>
@@ -1508,7 +1522,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>90</v>
       </c>
@@ -1528,7 +1542,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>90</v>
       </c>
@@ -1548,7 +1562,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>90</v>
       </c>
@@ -1568,7 +1582,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>90</v>
       </c>
@@ -1588,7 +1602,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>90</v>
       </c>
@@ -1608,7 +1622,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>90</v>
       </c>
@@ -1628,7 +1642,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>90</v>
       </c>
@@ -1648,7 +1662,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>90</v>
       </c>
@@ -1668,7 +1682,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>90</v>
       </c>
@@ -1688,7 +1702,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>110</v>
       </c>
@@ -1708,7 +1722,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>110</v>
       </c>
@@ -1728,7 +1742,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>110</v>
       </c>
@@ -1748,7 +1762,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>110</v>
       </c>
@@ -1768,7 +1782,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>110</v>
       </c>
@@ -1788,7 +1802,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>110</v>
       </c>
@@ -1808,7 +1822,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>110</v>
       </c>
@@ -1828,7 +1842,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>110</v>
       </c>
@@ -1848,7 +1862,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>117</v>
       </c>
@@ -1868,7 +1882,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>117</v>
       </c>
@@ -1888,7 +1902,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>117</v>
       </c>
@@ -1908,7 +1922,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>117</v>
       </c>
@@ -1928,7 +1942,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>117</v>
       </c>
@@ -1948,7 +1962,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>117</v>
       </c>
@@ -1968,7 +1982,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>117</v>
       </c>
@@ -1988,7 +2002,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>117</v>
       </c>
@@ -2008,7 +2022,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>117</v>
       </c>
@@ -2028,7 +2042,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>128</v>
       </c>
@@ -2048,7 +2062,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>128</v>
       </c>
@@ -2068,7 +2082,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>128</v>
       </c>
@@ -2088,7 +2102,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>128</v>
       </c>
@@ -2108,7 +2122,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>128</v>
       </c>
@@ -2128,7 +2142,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>128</v>
       </c>
@@ -2148,7 +2162,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>29</v>
       </c>

</xml_diff>

<commit_message>
Added spi_true, default indicators and many other edits
</commit_message>
<xml_diff>
--- a/data/reference_events.xlsx
+++ b/data/reference_events.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORK\IPC-HQ\RAAP - RISK ANALYSIS APPROACH\AFGHANISTAN\CLIMATOLOGICAL\pythonProject\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D22F69A0-B326-4CF7-B9A5-03472F00483A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E262420-9BE5-4A92-8033-C3E0145367DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11190" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="reference_events" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">reference_events!$A$1:$F$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">reference_events!$A$1:$F$85</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="137">
   <si>
     <t>country</t>
   </si>
@@ -811,15 +811,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:F85"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="7.42578125" customWidth="1"/>
     <col min="3" max="3" width="7.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="34" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -2182,7 +2182,348 @@
         <v>10</v>
       </c>
     </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D69" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E69" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F69" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D70" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E70" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F70" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D71" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E71" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F71" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D72" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E72" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F72" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D73" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E73" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F73" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D74" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E74" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F74" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C75" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D75" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E75" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F75" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D76" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E76" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F76" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D77" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E77" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F77" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D78" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="E78" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F78" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C79" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D79" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E79" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F79" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D80" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="E80" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F80" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C81" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D81" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E81" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F81" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="D82" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E82" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F82" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D83" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E83" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F83" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="C84" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D84" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="E84" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F84" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C85" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D85" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E85" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F85" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:F85" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Reference events for South Sudan added
</commit_message>
<xml_diff>
--- a/data/reference_events.xlsx
+++ b/data/reference_events.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORK\IPC-HQ\RAAP - RISK ANALYSIS APPROACH\AFGHANISTAN\CLIMATOLOGICAL\pythonProject\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E262420-9BE5-4A92-8033-C3E0145367DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AF6278D-24A4-49A2-8C04-289E1C7C0509}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11190" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="reference_events" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">reference_events!$A$1:$F$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">reference_events!$A$1:$F$104</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="672" uniqueCount="192">
   <si>
     <t>country</t>
   </si>
@@ -447,6 +447,171 @@
   </si>
   <si>
     <t>2025-09</t>
+  </si>
+  <si>
+    <t>1991-04</t>
+  </si>
+  <si>
+    <t>1992-08</t>
+  </si>
+  <si>
+    <t>Prolonged drought conditions (Northern &amp; Eastern regions)</t>
+  </si>
+  <si>
+    <t>1994-05</t>
+  </si>
+  <si>
+    <t>1994-08</t>
+  </si>
+  <si>
+    <t>Below-average rainfall (Northern zones)</t>
+  </si>
+  <si>
+    <t>1997-06</t>
+  </si>
+  <si>
+    <t>1997-09</t>
+  </si>
+  <si>
+    <t>Localised rainfall deficits – El Niño variability (Eastern regions)</t>
+  </si>
+  <si>
+    <t>2000-04</t>
+  </si>
+  <si>
+    <t>2000-07</t>
+  </si>
+  <si>
+    <t>Delayed onset and rainfall deficits (Northern &amp; Eastern regions)</t>
+  </si>
+  <si>
+    <t>2005-04</t>
+  </si>
+  <si>
+    <t>2006-08</t>
+  </si>
+  <si>
+    <t>Sustained multi-season rainfall deficits (multi-region)</t>
+  </si>
+  <si>
+    <t>2008-05</t>
+  </si>
+  <si>
+    <t>2009-08</t>
+  </si>
+  <si>
+    <t>Consecutive poor rainfall seasons (Greater Upper Nile)</t>
+  </si>
+  <si>
+    <t>2010-04</t>
+  </si>
+  <si>
+    <t>2011-09</t>
+  </si>
+  <si>
+    <t>Severe regional drought – Horn of Africa (Northern &amp; Eastern regions)</t>
+  </si>
+  <si>
+    <t>2012-05</t>
+  </si>
+  <si>
+    <t>2012-08</t>
+  </si>
+  <si>
+    <t>Seasonal rainfall deficits (Greater Upper Nile)</t>
+  </si>
+  <si>
+    <t>2014-04</t>
+  </si>
+  <si>
+    <t>2014-06</t>
+  </si>
+  <si>
+    <t>Erratic onset and rainfall deficits (Agro-pastoral zones)</t>
+  </si>
+  <si>
+    <t>2016-04</t>
+  </si>
+  <si>
+    <t>2016-06</t>
+  </si>
+  <si>
+    <t>Delayed onset of rainfall (Northern &amp; Eastern regions)</t>
+  </si>
+  <si>
+    <t>2017-05</t>
+  </si>
+  <si>
+    <t>2017-07</t>
+  </si>
+  <si>
+    <t>Localised rainfall deficits during food insecurity</t>
+  </si>
+  <si>
+    <t>2021-04</t>
+  </si>
+  <si>
+    <t>2021-06</t>
+  </si>
+  <si>
+    <t>Below-average onset rainfall (Eastern &amp; Northern regions)</t>
+  </si>
+  <si>
+    <t>Delayed onset and dry spells (Eastern Equatoria &amp; Jonglei)</t>
+  </si>
+  <si>
+    <t>2023-07</t>
+  </si>
+  <si>
+    <t>Above-average rainfall and flooding (Upper Nile, Jonglei, Unity)</t>
+  </si>
+  <si>
+    <t>2024-04</t>
+  </si>
+  <si>
+    <t>2024-06</t>
+  </si>
+  <si>
+    <t>Delayed onset and erratic rainfall (Greater Equatoria)</t>
+  </si>
+  <si>
+    <t>2024-07</t>
+  </si>
+  <si>
+    <t>2024-11</t>
+  </si>
+  <si>
+    <t>Widespread flooding linked to El Niño conditions</t>
+  </si>
+  <si>
+    <t>2025-04</t>
+  </si>
+  <si>
+    <t>2025-06</t>
+  </si>
+  <si>
+    <t>Early season rainfall deficits (localized drought risk)</t>
+  </si>
+  <si>
+    <t>2025-07</t>
+  </si>
+  <si>
+    <t>2025-10</t>
+  </si>
+  <si>
+    <t>Above-average rainfall and flood risk (Nile basin areas)</t>
+  </si>
+  <si>
+    <t>2026-04</t>
+  </si>
+  <si>
+    <t>2026-06</t>
+  </si>
+  <si>
+    <t>Delayed onset signals and rainfall deficits (early warning phase)</t>
+  </si>
+  <si>
+    <t>shock</t>
   </si>
 </sst>
 </file>
@@ -470,12 +635,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -505,10 +676,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -811,13 +983,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F85"/>
+  <dimension ref="A1:F112"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.42578125" customWidth="1"/>
-    <col min="3" max="3" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="34" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="37" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
@@ -2522,8 +2693,547 @@
         <v>15</v>
       </c>
     </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="D86" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="E86" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F86" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="D87" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="E87" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F87" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="D88" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="E88" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F88" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="C89" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="D89" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="E89" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F89" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="D90" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="E90" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F90" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C91" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="D91" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="E91" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F91" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="D92" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="E92" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F92" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="C93" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D93" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="E93" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F93" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="C94" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="D94" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="E94" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F94" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="C95" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="D95" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="E95" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F95" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C96" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="D96" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="E96" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F96" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="C97" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="D97" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="E97" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F97" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C98" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D98" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="E98" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F98" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="C99" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D99" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="E99" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F99" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="C100" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="D100" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="E100" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F100" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="C101" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D101" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="E101" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F101" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B102" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="C102" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="D102" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="E102" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F102" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="C103" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="D103" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="E103" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F103" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="C104" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="D104" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="E104" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F104" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B105" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C105" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D105" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="E105" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="F105" s="3" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B106" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C106" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D106" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="E106" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="F106" s="3" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B107" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="C107" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="D107" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="E107" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="F107" s="3" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B108" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C108" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="D108" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="E108" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="F108" s="3" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B109" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C109" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="D109" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="E109" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="F109" s="3" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="B110" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C110" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D110" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E110" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="F110" s="3" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="B111" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C111" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="D111" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="E111" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="F111" s="3" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="B112" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="C112" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D112" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E112" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="F112" s="3" t="s">
+        <v>191</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F85" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
No data category added, spi fully implemented for both drought and flood, descriptions adjusted and expander implemented
</commit_message>
<xml_diff>
--- a/data/reference_events.xlsx
+++ b/data/reference_events.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORK\IPC-HQ\RAAP - RISK ANALYSIS APPROACH\AFGHANISTAN\CLIMATOLOGICAL\pythonProject\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AF6278D-24A4-49A2-8C04-289E1C7C0509}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3714D3D7-4606-4112-AFFE-E2F6ED1FEFDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23190" yWindow="2040" windowWidth="15570" windowHeight="9315" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="reference_events" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">reference_events!$A$1:$F$104</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">reference_events!$A$1:$F$116</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="672" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="912" uniqueCount="256">
   <si>
     <t>country</t>
   </si>
@@ -203,9 +204,6 @@
     <t>Patel dam disaster</t>
   </si>
   <si>
-    <t>disaster</t>
-  </si>
-  <si>
     <t>2019-11</t>
   </si>
   <si>
@@ -218,9 +216,6 @@
     <t>Desert locust invasion</t>
   </si>
   <si>
-    <t>agriculture</t>
-  </si>
-  <si>
     <t>2020-01</t>
   </si>
   <si>
@@ -314,9 +309,6 @@
     <t>Sudan famine</t>
   </si>
   <si>
-    <t>food_security</t>
-  </si>
-  <si>
     <t>2005-01</t>
   </si>
   <si>
@@ -347,21 +339,12 @@
     <t>Famine declaration</t>
   </si>
   <si>
-    <t>Large-scale flooding</t>
-  </si>
-  <si>
     <t>2020-12</t>
   </si>
   <si>
-    <t>2021-01</t>
-  </si>
-  <si>
     <t>2025-12</t>
   </si>
   <si>
-    <t>Consecutive flood seasons</t>
-  </si>
-  <si>
     <t>2024-01</t>
   </si>
   <si>
@@ -560,9 +543,6 @@
     <t>Delayed onset and dry spells (Eastern Equatoria &amp; Jonglei)</t>
   </si>
   <si>
-    <t>2023-07</t>
-  </si>
-  <si>
     <t>Above-average rainfall and flooding (Upper Nile, Jonglei, Unity)</t>
   </si>
   <si>
@@ -575,9 +555,6 @@
     <t>Delayed onset and erratic rainfall (Greater Equatoria)</t>
   </si>
   <si>
-    <t>2024-07</t>
-  </si>
-  <si>
     <t>2024-11</t>
   </si>
   <si>
@@ -593,15 +570,9 @@
     <t>Early season rainfall deficits (localized drought risk)</t>
   </si>
   <si>
-    <t>2025-07</t>
-  </si>
-  <si>
     <t>2025-10</t>
   </si>
   <si>
-    <t>Above-average rainfall and flood risk (Nile basin areas)</t>
-  </si>
-  <si>
     <t>2026-04</t>
   </si>
   <si>
@@ -612,6 +583,228 @@
   </si>
   <si>
     <t>shock</t>
+  </si>
+  <si>
+    <t>2011-07</t>
+  </si>
+  <si>
+    <t>Post-independence tensions and localized conflict</t>
+  </si>
+  <si>
+    <t>2015-08</t>
+  </si>
+  <si>
+    <t>Civil war outbreak and widespread violence</t>
+  </si>
+  <si>
+    <t>2016-07</t>
+  </si>
+  <si>
+    <t>Resumption of conflict following Juba clashes</t>
+  </si>
+  <si>
+    <t>2018-09</t>
+  </si>
+  <si>
+    <t>Continued insecurity prior to peace agreement</t>
+  </si>
+  <si>
+    <t>Revitalized peace agreement period (reduced but persistent violence)</t>
+  </si>
+  <si>
+    <t>Sub-national intercommunal violence (Jonglei, Warrap, Lakes)</t>
+  </si>
+  <si>
+    <t>Escalation of localized armed clashes and cattle raiding</t>
+  </si>
+  <si>
+    <t>Continued intercommunal violence and localized insecurity</t>
+  </si>
+  <si>
+    <t>Persistent sub-national conflict and political tensions</t>
+  </si>
+  <si>
+    <t>2025-01</t>
+  </si>
+  <si>
+    <t>Ongoing localized conflict and access constraints</t>
+  </si>
+  <si>
+    <t>Continued insecurity (early warning / evolving context)</t>
+  </si>
+  <si>
+    <t>1990-10</t>
+  </si>
+  <si>
+    <t>Seasonal flooding along Nile and Sobat river basins</t>
+  </si>
+  <si>
+    <t>1998-11</t>
+  </si>
+  <si>
+    <t>2007-10</t>
+  </si>
+  <si>
+    <t>Severe floods affecting large parts of the country</t>
+  </si>
+  <si>
+    <t>2017-10</t>
+  </si>
+  <si>
+    <t>Extreme and prolonged flooding across multiple states</t>
+  </si>
+  <si>
+    <t>Continued multi-year flooding crisis</t>
+  </si>
+  <si>
+    <t>Persistent flooding in Nile basin and Sudd wetlands</t>
+  </si>
+  <si>
+    <t>2026-10</t>
+  </si>
+  <si>
+    <t>drought</t>
+  </si>
+  <si>
+    <t>flood</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Start</t>
+  </si>
+  <si>
+    <t>End</t>
+  </si>
+  <si>
+    <t>Event description</t>
+  </si>
+  <si>
+    <t>Spatial focus</t>
+  </si>
+  <si>
+    <t>Notes / Use in validation</t>
+  </si>
+  <si>
+    <t>Jul</t>
+  </si>
+  <si>
+    <t>Oct</t>
+  </si>
+  <si>
+    <t>Nile &amp; Sobat basins</t>
+  </si>
+  <si>
+    <t>Nov</t>
+  </si>
+  <si>
+    <t>Widespread</t>
+  </si>
+  <si>
+    <t>Extreme benchmark event</t>
+  </si>
+  <si>
+    <t>Nationwide</t>
+  </si>
+  <si>
+    <t>High-impact flood year</t>
+  </si>
+  <si>
+    <t>Sudd wetlands</t>
+  </si>
+  <si>
+    <t>Dec</t>
+  </si>
+  <si>
+    <t>Start of multi-year flood crisis</t>
+  </si>
+  <si>
+    <t>Severe, widespread flooding (East Africa floods)</t>
+  </si>
+  <si>
+    <t>Nile basin &amp; Sudd</t>
+  </si>
+  <si>
+    <t>Long-duration flood conditions</t>
+  </si>
+  <si>
+    <t>Eastern regions</t>
+  </si>
+  <si>
+    <t>Above-average rainfall and elevated flood risk</t>
+  </si>
+  <si>
+    <t>Nile basin areas</t>
+  </si>
+  <si>
+    <t>Flood-prone areas</t>
+  </si>
+  <si>
+    <t>Jun</t>
+  </si>
+  <si>
+    <t>Baseline seasonal flooding (non-extreme reference)</t>
+  </si>
+  <si>
+    <t>Major flooding linked to El Niño conditions</t>
+  </si>
+  <si>
+    <t>Localized flooding in Sudd wetlands</t>
+  </si>
+  <si>
+    <t>Secondary / sensitivity testing</t>
+  </si>
+  <si>
+    <t>May</t>
+  </si>
+  <si>
+    <t>Very early onset + peak flood year</t>
+  </si>
+  <si>
+    <t>Persistence validation</t>
+  </si>
+  <si>
+    <t>Strong regional signal</t>
+  </si>
+  <si>
+    <t>Climate-driven validation</t>
+  </si>
+  <si>
+    <t>Early warning / monitoring</t>
+  </si>
+  <si>
+    <t>Seasonal flood risk (evolving conditions)</t>
+  </si>
+  <si>
+    <t>Forward-looking application</t>
+  </si>
+  <si>
+    <t>event_description</t>
+  </si>
+  <si>
+    <t>event_type</t>
+  </si>
+  <si>
+    <t>category</t>
+  </si>
+  <si>
+    <t>1990-06</t>
+  </si>
+  <si>
+    <t>1998-06</t>
+  </si>
+  <si>
+    <t>2007-06</t>
+  </si>
+  <si>
+    <t>2019-06</t>
+  </si>
+  <si>
+    <t>2020-05</t>
+  </si>
+  <si>
+    <t>2022-06</t>
   </si>
 </sst>
 </file>
@@ -649,7 +842,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -672,15 +865,38 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -983,12 +1199,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F112"/>
+  <dimension ref="A1:F128"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="37" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="56.140625" customWidth="1"/>
     <col min="5" max="5" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
@@ -1027,29 +1243,29 @@
         <v>9</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>10</v>
+        <v>209</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" s="5" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1127,7 +1343,7 @@
         <v>28</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>10</v>
+        <v>209</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>10</v>
@@ -1147,29 +1363,29 @@
         <v>30</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>10</v>
+        <v>209</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="D9" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="E9" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F9" s="1" t="s">
+      <c r="E9" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="F9" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1186,8 +1402,8 @@
       <c r="D10" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E10" s="1" t="s">
-        <v>10</v>
+      <c r="E10" s="5" t="s">
+        <v>208</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>10</v>
@@ -1226,8 +1442,8 @@
       <c r="D12" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="E12" s="1" t="s">
-        <v>10</v>
+      <c r="E12" s="5" t="s">
+        <v>208</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>10</v>
@@ -1246,8 +1462,8 @@
       <c r="D13" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="E13" s="1" t="s">
-        <v>10</v>
+      <c r="E13" s="5" t="s">
+        <v>208</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>10</v>
@@ -1266,8 +1482,8 @@
       <c r="D14" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E14" s="1" t="s">
-        <v>10</v>
+      <c r="E14" s="5" t="s">
+        <v>208</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>10</v>
@@ -1286,8 +1502,8 @@
       <c r="D15" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="E15" s="1" t="s">
-        <v>10</v>
+      <c r="E15" s="5" t="s">
+        <v>208</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>10</v>
@@ -1307,29 +1523,29 @@
         <v>52</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>10</v>
+        <v>209</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
+      <c r="A17" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="D17" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="E17" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="F17" s="1" t="s">
+      <c r="E17" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="F17" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1338,16 +1554,16 @@
         <v>29</v>
       </c>
       <c r="B18" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D18" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C18" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>55</v>
+      <c r="E18" s="5" t="s">
+        <v>208</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>10</v>
@@ -1358,16 +1574,16 @@
         <v>29</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>20</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>208</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>10</v>
@@ -1378,16 +1594,16 @@
         <v>29</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D20" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C20" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>10</v>
+      <c r="E20" s="5" t="s">
+        <v>208</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>10</v>
@@ -1398,7 +1614,7 @@
         <v>29</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>27</v>
@@ -1407,7 +1623,7 @@
         <v>30</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>10</v>
+        <v>209</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>10</v>
@@ -1418,53 +1634,53 @@
         <v>29</v>
       </c>
       <c r="B22" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D22" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="E22" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="B23" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="E22" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="C23" s="1" t="s">
+      <c r="C23" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="D23" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="E23" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F23" s="1" t="s">
+      <c r="E23" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="F23" s="5" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B24" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="C24" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D24" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>72</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>40</v>
@@ -1475,7 +1691,7 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>11</v>
@@ -1484,30 +1700,30 @@
         <v>12</v>
       </c>
       <c r="D25" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F25" s="1" t="s">
         <v>73</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>43</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="E26" s="1" t="s">
-        <v>10</v>
+      <c r="E26" s="5" t="s">
+        <v>208</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>10</v>
@@ -1515,7 +1731,7 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>45</v>
@@ -1524,10 +1740,10 @@
         <v>46</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>15</v>
@@ -1535,7 +1751,7 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>48</v>
@@ -1544,90 +1760,90 @@
         <v>49</v>
       </c>
       <c r="D28" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="D29" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="E28" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F29" s="1" t="s">
+      <c r="E29" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="F29" s="5" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C30" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D30" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="D30" s="1" t="s">
-        <v>82</v>
-      </c>
       <c r="E30" s="1" t="s">
-        <v>10</v>
+        <v>209</v>
       </c>
       <c r="F30" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="B31" s="1" t="s">
+      <c r="A31" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B31" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="C31" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D31" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="E31" s="1" t="s">
+      <c r="D31" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="E31" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="F31" s="1" t="s">
+      <c r="F31" s="5" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B32" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D32" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C32" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>86</v>
-      </c>
       <c r="E32" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F32" s="1" t="s">
         <v>15</v>
@@ -1635,16 +1851,16 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>14</v>
@@ -1655,7 +1871,7 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>26</v>
@@ -1664,47 +1880,47 @@
         <v>27</v>
       </c>
       <c r="D34" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D35" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="E34" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="E35" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="F35" s="1" t="s">
+      <c r="E35" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="F35" s="5" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B36" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B36" s="1" t="s">
-        <v>93</v>
-      </c>
       <c r="C36" s="1" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>40</v>
@@ -1715,7 +1931,7 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>43</v>
@@ -1724,7 +1940,7 @@
         <v>17</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="E37" s="1" t="s">
         <v>40</v>
@@ -1735,19 +1951,19 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>51</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F38" s="1" t="s">
         <v>15</v>
@@ -1755,7 +1971,7 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>45</v>
@@ -1764,10 +1980,10 @@
         <v>46</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
+      </c>
+      <c r="E39" s="5" t="s">
+        <v>208</v>
       </c>
       <c r="F39" s="1" t="s">
         <v>10</v>
@@ -1775,7 +1991,7 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>48</v>
@@ -1784,50 +2000,50 @@
         <v>49</v>
       </c>
       <c r="D40" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E40" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="B41" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="E40" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="F40" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="D41" s="1" t="s">
+      <c r="C41" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="D41" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="E41" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F41" s="1" t="s">
-        <v>10</v>
+      <c r="E41" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="F41" s="5" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>61</v>
+        <v>31</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>104</v>
+        <v>32</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="E42" s="1" t="s">
-        <v>10</v>
+        <v>33</v>
+      </c>
+      <c r="E42" s="5" t="s">
+        <v>208</v>
       </c>
       <c r="F42" s="1" t="s">
         <v>10</v>
@@ -1835,59 +2051,59 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>105</v>
       </c>
       <c r="C43" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D43" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="D43" s="1" t="s">
+      <c r="E43" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="D44" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="E43" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F43" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="D44" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="F44" s="1" t="s">
-        <v>15</v>
+      <c r="E44" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="F44" s="5" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D45" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="B45" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C45" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D45" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>10</v>
+      <c r="E45" s="5" t="s">
+        <v>208</v>
       </c>
       <c r="F45" s="1" t="s">
         <v>10</v>
@@ -1895,59 +2111,59 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>111</v>
+        <v>50</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>112</v>
+        <v>52</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>10</v>
+        <v>209</v>
       </c>
       <c r="F46" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A47" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="B47" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C47" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D47" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="E47" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="F47" s="1" t="s">
+      <c r="A47" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C47" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D47" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E47" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="F47" s="5" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>115</v>
+        <v>59</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="E48" s="1" t="s">
-        <v>10</v>
+        <v>61</v>
+      </c>
+      <c r="E48" s="5" t="s">
+        <v>208</v>
       </c>
       <c r="F48" s="1" t="s">
         <v>10</v>
@@ -1955,59 +2171,59 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>10</v>
+        <v>209</v>
       </c>
       <c r="F49" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A50" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="B50" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C50" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D50" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="E50" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="F50" s="1" t="s">
+      <c r="A50" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B50" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="D50" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E50" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="F50" s="5" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>61</v>
+        <v>113</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>62</v>
+        <v>114</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="E51" s="1" t="s">
-        <v>10</v>
+        <v>115</v>
+      </c>
+      <c r="E51" s="5" t="s">
+        <v>208</v>
       </c>
       <c r="F51" s="1" t="s">
         <v>10</v>
@@ -2015,19 +2231,19 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>64</v>
+        <v>43</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E52" s="1" t="s">
-        <v>10</v>
+        <v>44</v>
+      </c>
+      <c r="E52" s="5" t="s">
+        <v>208</v>
       </c>
       <c r="F52" s="1" t="s">
         <v>10</v>
@@ -2035,19 +2251,19 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C53" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="B53" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C53" s="1" t="s">
+      <c r="D53" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="D53" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="E53" s="1" t="s">
-        <v>10</v>
+      <c r="E53" s="5" t="s">
+        <v>208</v>
       </c>
       <c r="F53" s="1" t="s">
         <v>10</v>
@@ -2055,59 +2271,59 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>119</v>
+        <v>50</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>120</v>
+        <v>51</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>121</v>
+        <v>52</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>10</v>
+        <v>209</v>
       </c>
       <c r="F54" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A55" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="B55" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C55" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D55" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="E55" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F55" s="1" t="s">
+      <c r="A55" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B55" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C55" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E55" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="F55" s="5" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>122</v>
+        <v>59</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>123</v>
+        <v>60</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="E56" s="1" t="s">
-        <v>10</v>
+        <v>61</v>
+      </c>
+      <c r="E56" s="5" t="s">
+        <v>208</v>
       </c>
       <c r="F56" s="1" t="s">
         <v>10</v>
@@ -2115,79 +2331,79 @@
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>50</v>
+        <v>119</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>51</v>
+        <v>120</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>52</v>
+        <v>121</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>60</v>
+        <v>209</v>
       </c>
       <c r="F58" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A59" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="B59" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="C59" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D59" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="E59" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F59" s="1" t="s">
+      <c r="A59" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="B59" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C59" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D59" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="E59" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="F59" s="5" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>126</v>
+        <v>91</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F60" s="1" t="s">
         <v>15</v>
@@ -2195,139 +2411,139 @@
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>64</v>
+        <v>43</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>30</v>
+        <v>124</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>69</v>
+        <v>50</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>8</v>
+        <v>78</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>91</v>
+        <v>125</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>114</v>
+        <v>14</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E63" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="F63" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="B64" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="C64" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D64" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="B63" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="C63" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="D63" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="E63" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="F63" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A64" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="B64" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C64" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D64" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="E64" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="F64" s="1" t="s">
+      <c r="E64" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="F64" s="5" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
-        <v>128</v>
+        <v>29</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>50</v>
+        <v>129</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>80</v>
+        <v>130</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>131</v>
+        <v>65</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>14</v>
+        <v>209</v>
       </c>
       <c r="F65" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B66" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C66" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D66" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E66" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F66" s="5" t="s">
         <v>15</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A66" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="B66" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="C66" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="E66" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F66" s="1" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
-        <v>128</v>
+        <v>29</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>133</v>
+        <v>34</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>134</v>
+        <v>36</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>99</v>
+        <v>10</v>
       </c>
       <c r="F67" s="1" t="s">
         <v>15</v>
@@ -2338,19 +2554,19 @@
         <v>29</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>135</v>
+        <v>41</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>136</v>
+        <v>42</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>67</v>
+        <v>33</v>
       </c>
       <c r="E68" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
@@ -2358,13 +2574,13 @@
         <v>29</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="E69" s="1" t="s">
         <v>10</v>
@@ -2378,13 +2594,13 @@
         <v>29</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="E70" s="1" t="s">
         <v>10</v>
@@ -2398,10 +2614,10 @@
         <v>29</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D71" s="1" t="s">
         <v>33</v>
@@ -2418,13 +2634,13 @@
         <v>29</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>17</v>
+        <v>60</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="E72" s="1" t="s">
         <v>10</v>
@@ -2435,16 +2651,16 @@
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
-        <v>29</v>
+        <v>66</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>45</v>
+        <v>67</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="E73" s="1" t="s">
         <v>10</v>
@@ -2455,13 +2671,13 @@
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
-        <v>29</v>
+        <v>66</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>49</v>
+        <v>74</v>
       </c>
       <c r="D74" s="1" t="s">
         <v>33</v>
@@ -2475,16 +2691,16 @@
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
-        <v>29</v>
+        <v>66</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="E75" s="1" t="s">
         <v>10</v>
@@ -2495,16 +2711,16 @@
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
-        <v>68</v>
+        <v>104</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>69</v>
+        <v>31</v>
       </c>
       <c r="C76" s="1" t="s">
         <v>32</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E76" s="1" t="s">
         <v>10</v>
@@ -2515,16 +2731,16 @@
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
-        <v>68</v>
+        <v>104</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>43</v>
+        <v>109</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>76</v>
+        <v>49</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>33</v>
+        <v>110</v>
       </c>
       <c r="E77" s="1" t="s">
         <v>10</v>
@@ -2535,16 +2751,16 @@
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
-        <v>68</v>
+        <v>104</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>81</v>
+        <v>61</v>
       </c>
       <c r="E78" s="1" t="s">
         <v>10</v>
@@ -2555,16 +2771,16 @@
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B79" s="1" t="s">
         <v>31</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>32</v>
+        <v>112</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E79" s="1" t="s">
         <v>10</v>
@@ -2575,16 +2791,16 @@
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>115</v>
+        <v>43</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>116</v>
+        <v>44</v>
       </c>
       <c r="E80" s="1" t="s">
         <v>10</v>
@@ -2595,16 +2811,16 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>61</v>
+        <v>116</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>62</v>
+        <v>117</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>63</v>
+        <v>118</v>
       </c>
       <c r="E81" s="1" t="s">
         <v>10</v>
@@ -2615,16 +2831,16 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>31</v>
+        <v>59</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>118</v>
+        <v>60</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>36</v>
+        <v>61</v>
       </c>
       <c r="E82" s="1" t="s">
         <v>10</v>
@@ -2635,79 +2851,79 @@
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
-        <v>117</v>
+        <v>88</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>43</v>
+        <v>131</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>17</v>
+        <v>132</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="E83" s="1" t="s">
-        <v>10</v>
+        <v>133</v>
+      </c>
+      <c r="E83" s="5" t="s">
+        <v>208</v>
       </c>
       <c r="F83" s="1" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
-        <v>117</v>
+        <v>88</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>123</v>
+        <v>135</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="E84" s="1" t="s">
-        <v>10</v>
+        <v>136</v>
+      </c>
+      <c r="E84" s="5" t="s">
+        <v>208</v>
       </c>
       <c r="F84" s="1" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
-        <v>117</v>
+        <v>88</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>61</v>
+        <v>137</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>62</v>
+        <v>138</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="E85" s="1" t="s">
-        <v>10</v>
+        <v>139</v>
+      </c>
+      <c r="E85" s="5" t="s">
+        <v>208</v>
       </c>
       <c r="F85" s="1" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="E86" s="1" t="s">
-        <v>10</v>
+        <v>142</v>
+      </c>
+      <c r="E86" s="5" t="s">
+        <v>208</v>
       </c>
       <c r="F86" s="1" t="s">
         <v>10</v>
@@ -2715,19 +2931,19 @@
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="E87" s="1" t="s">
-        <v>10</v>
+        <v>145</v>
+      </c>
+      <c r="E87" s="5" t="s">
+        <v>208</v>
       </c>
       <c r="F87" s="1" t="s">
         <v>10</v>
@@ -2735,19 +2951,19 @@
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="E88" s="1" t="s">
-        <v>10</v>
+        <v>148</v>
+      </c>
+      <c r="E88" s="5" t="s">
+        <v>208</v>
       </c>
       <c r="F88" s="1" t="s">
         <v>10</v>
@@ -2755,19 +2971,19 @@
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="E89" s="1" t="s">
-        <v>10</v>
+        <v>151</v>
+      </c>
+      <c r="E89" s="5" t="s">
+        <v>208</v>
       </c>
       <c r="F89" s="1" t="s">
         <v>10</v>
@@ -2775,19 +2991,19 @@
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="E90" s="1" t="s">
-        <v>10</v>
+        <v>154</v>
+      </c>
+      <c r="E90" s="5" t="s">
+        <v>208</v>
       </c>
       <c r="F90" s="1" t="s">
         <v>10</v>
@@ -2795,19 +3011,19 @@
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="E91" s="1" t="s">
-        <v>10</v>
+        <v>157</v>
+      </c>
+      <c r="E91" s="5" t="s">
+        <v>208</v>
       </c>
       <c r="F91" s="1" t="s">
         <v>10</v>
@@ -2815,19 +3031,19 @@
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="E92" s="1" t="s">
-        <v>10</v>
+        <v>160</v>
+      </c>
+      <c r="E92" s="5" t="s">
+        <v>208</v>
       </c>
       <c r="F92" s="1" t="s">
         <v>10</v>
@@ -2835,19 +3051,19 @@
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="E93" s="1" t="s">
-        <v>10</v>
+        <v>163</v>
+      </c>
+      <c r="E93" s="5" t="s">
+        <v>208</v>
       </c>
       <c r="F93" s="1" t="s">
         <v>10</v>
@@ -2855,19 +3071,19 @@
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="D94" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="E94" s="1" t="s">
-        <v>10</v>
+        <v>166</v>
+      </c>
+      <c r="E94" s="5" t="s">
+        <v>208</v>
       </c>
       <c r="F94" s="1" t="s">
         <v>10</v>
@@ -2875,365 +3091,1222 @@
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>164</v>
+        <v>127</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>165</v>
+        <v>60</v>
       </c>
       <c r="D95" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="E95" s="1" t="s">
-        <v>10</v>
+        <v>167</v>
+      </c>
+      <c r="E95" s="5" t="s">
+        <v>208</v>
       </c>
       <c r="F95" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A96" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="B96" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="C96" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="D96" s="1" t="s">
+      <c r="A96" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="B96" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="E96" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F96" s="1" t="s">
+      <c r="C96" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="D96" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="E96" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="F96" s="5" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A97" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="B97" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="C97" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="D97" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="E97" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F97" s="1" t="s">
+      <c r="A97" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="B97" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="C97" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="D97" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="E97" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="F97" s="5" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A98" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="B98" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="C98" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D98" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="E98" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F98" s="1" t="s">
+      <c r="A98" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="B98" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="C98" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="D98" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="E98" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="F98" s="5" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A99" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="B99" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="C99" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="D99" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="E99" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F99" s="1" t="s">
-        <v>10</v>
+      <c r="A99" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B99" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C99" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D99" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E99" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="F99" s="3" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A100" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="B100" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="C100" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="D100" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="E100" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F100" s="1" t="s">
-        <v>10</v>
+      <c r="A100" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B100" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="C100" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="D100" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="E100" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="F100" s="3" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A101" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="B101" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="C101" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="D101" s="1" t="s">
+      <c r="A101" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B101" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C101" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="D101" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E101" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="F101" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="E101" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F101" s="1" t="s">
-        <v>10</v>
-      </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A102" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="B102" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="C102" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="D102" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="E102" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F102" s="1" t="s">
-        <v>10</v>
+      <c r="A102" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="B102" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C102" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D102" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E102" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="F102" s="3" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A103" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="B103" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="C103" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="D103" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="E103" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F103" s="1" t="s">
-        <v>10</v>
+      <c r="A103" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B103" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C103" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D103" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E103" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="F103" s="3" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A104" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="B104" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="C104" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="D104" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="E104" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F104" s="1" t="s">
-        <v>10</v>
+      <c r="A104" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B104" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C104" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="D104" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="E104" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="F104" s="3" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" s="3" t="s">
-        <v>90</v>
+        <v>122</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>97</v>
+        <v>127</v>
       </c>
       <c r="C105" s="3" t="s">
-        <v>51</v>
+        <v>64</v>
       </c>
       <c r="D105" s="3" t="s">
-        <v>98</v>
+        <v>128</v>
       </c>
       <c r="E105" s="3" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F105" s="3" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A106" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B106" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="C106" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D106" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="E106" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F106" s="4" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A107" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C107" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="D107" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="E107" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F107" s="4" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A108" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B108" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="C108" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D108" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="E108" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F108" s="4" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A109" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C109" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="D109" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="E109" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F109" s="4" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A110" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B110" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="C110" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="D110" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="E110" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F110" s="4" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A111" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B111" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C111" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D111" s="4" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A106" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="B106" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C106" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="D106" s="3" t="s">
+      <c r="E111" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F111" s="4" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A112" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B112" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C112" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="D112" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="E112" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F112" s="4" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A113" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B113" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C113" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D113" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="E113" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F113" s="4" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A114" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B114" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C114" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D114" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="E114" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F114" s="4" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A115" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B115" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="C115" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="D115" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="E115" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F115" s="4" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A116" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B116" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C116" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D116" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="E116" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F116" s="4" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>88</v>
+      </c>
+      <c r="B117" t="s">
+        <v>250</v>
+      </c>
+      <c r="C117" t="s">
+        <v>198</v>
+      </c>
+      <c r="D117" t="s">
+        <v>199</v>
+      </c>
+      <c r="E117" t="s">
+        <v>209</v>
+      </c>
+      <c r="F117" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>88</v>
+      </c>
+      <c r="B118" t="s">
+        <v>251</v>
+      </c>
+      <c r="C118" t="s">
+        <v>200</v>
+      </c>
+      <c r="D118" t="s">
+        <v>236</v>
+      </c>
+      <c r="E118" t="s">
+        <v>209</v>
+      </c>
+      <c r="F118" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>88</v>
+      </c>
+      <c r="B119" t="s">
+        <v>252</v>
+      </c>
+      <c r="C119" t="s">
+        <v>201</v>
+      </c>
+      <c r="D119" t="s">
+        <v>202</v>
+      </c>
+      <c r="E119" t="s">
+        <v>209</v>
+      </c>
+      <c r="F119" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>88</v>
+      </c>
+      <c r="B120" t="s">
+        <v>162</v>
+      </c>
+      <c r="C120" t="s">
+        <v>203</v>
+      </c>
+      <c r="D120" t="s">
+        <v>237</v>
+      </c>
+      <c r="E120" t="s">
+        <v>209</v>
+      </c>
+      <c r="F120" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>88</v>
+      </c>
+      <c r="B121" t="s">
+        <v>253</v>
+      </c>
+      <c r="C121" t="s">
+        <v>78</v>
+      </c>
+      <c r="D121" t="s">
+        <v>204</v>
+      </c>
+      <c r="E121" t="s">
+        <v>209</v>
+      </c>
+      <c r="F121" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>88</v>
+      </c>
+      <c r="B122" t="s">
+        <v>254</v>
+      </c>
+      <c r="C122" t="s">
         <v>100</v>
       </c>
-      <c r="E106" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="F106" s="3" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A107" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="B107" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="C107" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="D107" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="E107" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="F107" s="3" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A108" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="B108" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C108" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="D108" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="E108" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="F108" s="3" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A109" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="B109" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="C109" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="D109" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="E109" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="F109" s="3" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A110" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="B110" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="C110" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D110" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="E110" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="F110" s="3" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A111" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="B111" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="C111" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="D111" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="E111" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="F111" s="3" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A112" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="B112" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="C112" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="D112" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="E112" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="F112" s="3" t="s">
-        <v>191</v>
+      <c r="D122" t="s">
+        <v>227</v>
+      </c>
+      <c r="E122" t="s">
+        <v>209</v>
+      </c>
+      <c r="F122" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>88</v>
+      </c>
+      <c r="B123" t="s">
+        <v>165</v>
+      </c>
+      <c r="C123" t="s">
+        <v>20</v>
+      </c>
+      <c r="D123" t="s">
+        <v>205</v>
+      </c>
+      <c r="E123" t="s">
+        <v>209</v>
+      </c>
+      <c r="F123" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>88</v>
+      </c>
+      <c r="B124" t="s">
+        <v>255</v>
+      </c>
+      <c r="C124" t="s">
+        <v>83</v>
+      </c>
+      <c r="D124" t="s">
+        <v>206</v>
+      </c>
+      <c r="E124" t="s">
+        <v>209</v>
+      </c>
+      <c r="F124" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>88</v>
+      </c>
+      <c r="B125" t="s">
+        <v>60</v>
+      </c>
+      <c r="C125" t="s">
+        <v>24</v>
+      </c>
+      <c r="D125" t="s">
+        <v>168</v>
+      </c>
+      <c r="E125" t="s">
+        <v>209</v>
+      </c>
+      <c r="F125" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>88</v>
+      </c>
+      <c r="B126" t="s">
+        <v>170</v>
+      </c>
+      <c r="C126" t="s">
+        <v>172</v>
+      </c>
+      <c r="D126" t="s">
+        <v>173</v>
+      </c>
+      <c r="E126" t="s">
+        <v>209</v>
+      </c>
+      <c r="F126" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>88</v>
+      </c>
+      <c r="B127" t="s">
+        <v>175</v>
+      </c>
+      <c r="C127" t="s">
+        <v>177</v>
+      </c>
+      <c r="D127" t="s">
+        <v>231</v>
+      </c>
+      <c r="E127" t="s">
+        <v>209</v>
+      </c>
+      <c r="F127" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>88</v>
+      </c>
+      <c r="B128" t="s">
+        <v>179</v>
+      </c>
+      <c r="C128" t="s">
+        <v>207</v>
+      </c>
+      <c r="D128" t="s">
+        <v>245</v>
+      </c>
+      <c r="E128" t="s">
+        <v>209</v>
+      </c>
+      <c r="F128" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9190875E-349E-419D-BC35-080EF951BF12}">
+  <dimension ref="A1:F29"/>
+  <sheetFormatPr defaultColWidth="125.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="58.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="44.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="7">
+        <v>1990</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="7">
+        <v>1998</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="7">
+        <v>2007</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="7">
+        <v>2017</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="7">
+        <v>2019</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="7">
+        <v>2020</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="7">
+        <v>2021</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="7">
+        <v>2022</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="7">
+        <v>2023</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="7">
+        <v>2024</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="7">
+        <v>2025</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="7">
+        <v>2026</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A18" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A19" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>251</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A20" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>252</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A21" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A22" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>253</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A23" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>254</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A24" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A25" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>255</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A26" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="E26" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A27" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="E27" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A28" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="E28" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A29" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="E29" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
alps, vci,morbidity and other major changes made
</commit_message>
<xml_diff>
--- a/data/reference_events.xlsx
+++ b/data/reference_events.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORK\IPC-HQ\RAAP - RISK ANALYSIS APPROACH\AFGHANISTAN\CLIMATOLOGICAL\pythonProject\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35BECA19-A253-46BB-891E-1D4C724345F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{202C01CD-66F4-4CAA-8DAE-117932B7E8B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">reference_events!$A$1:$F$113</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">reference_events!$A$1:$F$220</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="942" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1463" uniqueCount="427">
   <si>
     <t>country</t>
   </si>
@@ -829,6 +829,495 @@
   </si>
   <si>
     <t>Protracted displacement crisis â€“ chronic vulnerability</t>
+  </si>
+  <si>
+    <t>2000-01</t>
+  </si>
+  <si>
+    <t>drought/economic</t>
+  </si>
+  <si>
+    <t>2008-09</t>
+  </si>
+  <si>
+    <t>2012-03</t>
+  </si>
+  <si>
+    <t>2015-10</t>
+  </si>
+  <si>
+    <t>2016-10</t>
+  </si>
+  <si>
+    <t>2017-11</t>
+  </si>
+  <si>
+    <t>2017-09</t>
+  </si>
+  <si>
+    <t>policy</t>
+  </si>
+  <si>
+    <t>recovery</t>
+  </si>
+  <si>
+    <t>pest</t>
+  </si>
+  <si>
+    <t>2021-09</t>
+  </si>
+  <si>
+    <t>2022-07</t>
+  </si>
+  <si>
+    <t>2022-10</t>
+  </si>
+  <si>
+    <t>2022-09</t>
+  </si>
+  <si>
+    <t>2001-03</t>
+  </si>
+  <si>
+    <t>2002-09</t>
+  </si>
+  <si>
+    <t>2003-02</t>
+  </si>
+  <si>
+    <t>2004-10</t>
+  </si>
+  <si>
+    <t>2006-03</t>
+  </si>
+  <si>
+    <t>2006-10</t>
+  </si>
+  <si>
+    <t>2008-10</t>
+  </si>
+  <si>
+    <t>2009-03</t>
+  </si>
+  <si>
+    <t>La Niña</t>
+  </si>
+  <si>
+    <t>2011-10</t>
+  </si>
+  <si>
+    <t>2010-07</t>
+  </si>
+  <si>
+    <t>2011-04</t>
+  </si>
+  <si>
+    <t>2012-10</t>
+  </si>
+  <si>
+    <t>2013-05</t>
+  </si>
+  <si>
+    <t>2014-10</t>
+  </si>
+  <si>
+    <t>2015-05</t>
+  </si>
+  <si>
+    <t>2015-09</t>
+  </si>
+  <si>
+    <t>2016-05</t>
+  </si>
+  <si>
+    <t>2017-03</t>
+  </si>
+  <si>
+    <t>2018-03</t>
+  </si>
+  <si>
+    <t>2018-06</t>
+  </si>
+  <si>
+    <t>2018-10</t>
+  </si>
+  <si>
+    <t>2019-10</t>
+  </si>
+  <si>
+    <t>2020-09</t>
+  </si>
+  <si>
+    <t>2022-03</t>
+  </si>
+  <si>
+    <t>2024-05</t>
+  </si>
+  <si>
+    <t>2024-03</t>
+  </si>
+  <si>
+    <t>2025-03</t>
+  </si>
+  <si>
+    <t>2026-02</t>
+  </si>
+  <si>
+    <t>2026-03</t>
+  </si>
+  <si>
+    <t>2001-01</t>
+  </si>
+  <si>
+    <t>Escalation of cattle rustling and intercommunal violence in northern Kenya disrupting livelihoods and livestock trade</t>
+  </si>
+  <si>
+    <t>conflict</t>
+  </si>
+  <si>
+    <t>Increased intercommunal conflict over pasture and water resources in ASAL counties during prolonged drought</t>
+  </si>
+  <si>
+    <t>Post-election violence causing over 1,100 deaths, large-scale displacement and widespread market disruption</t>
+  </si>
+  <si>
+    <t>political violence</t>
+  </si>
+  <si>
+    <t>2008-06</t>
+  </si>
+  <si>
+    <t>Humanitarian response to post-election displacement with major livelihood and food security impacts</t>
+  </si>
+  <si>
+    <t>displacement</t>
+  </si>
+  <si>
+    <t>Kenya Defence Forces intervention in Somalia (Operation Linda Nchi) followed by increased cross-border security incidents</t>
+  </si>
+  <si>
+    <t>2012-01</t>
+  </si>
+  <si>
+    <t>Intensified Al-Shabaab attacks in northeastern Kenya affecting trade, transport and humanitarian operations</t>
+  </si>
+  <si>
+    <t>terrorism</t>
+  </si>
+  <si>
+    <t>2013-09</t>
+  </si>
+  <si>
+    <t>Westgate Shopping Mall terrorist attack in Nairobi leading to heightened national security measures</t>
+  </si>
+  <si>
+    <t>Mpeketoni attacks in Lamu County resulting in prolonged insecurity along the coast</t>
+  </si>
+  <si>
+    <t>Escalation of terrorist attacks in northeastern Kenya disrupting livelihoods and service delivery</t>
+  </si>
+  <si>
+    <t>2015-04</t>
+  </si>
+  <si>
+    <t>Garissa University terrorist attack leading to strengthened national security operations</t>
+  </si>
+  <si>
+    <t>Continued insecurity along the Somalia border affecting humanitarian access and cross-border trade</t>
+  </si>
+  <si>
+    <t>Increased intercommunal conflict over grazing resources in Turkana, Baringo, West Pokot and Samburu</t>
+  </si>
+  <si>
+    <t>2017-08</t>
+  </si>
+  <si>
+    <t>General election-related tensions and localized violence during repeat presidential election period</t>
+  </si>
+  <si>
+    <t>Persistent communal conflict and livestock raids across northwestern Kenya</t>
+  </si>
+  <si>
+    <t>DusitD2 terrorist attack in Nairobi resulting in increased national security operations</t>
+  </si>
+  <si>
+    <t>Increased insecurity and intercommunal conflict in parts of ASAL counties driven by resource competition</t>
+  </si>
+  <si>
+    <t>2021-01</t>
+  </si>
+  <si>
+    <t>Continued Al-Shabaab cross-border attacks and IED incidents affecting northeastern counties</t>
+  </si>
+  <si>
+    <t>General election conducted with localized security incidents but limited nationwide disruption</t>
+  </si>
+  <si>
+    <t>Continued insecurity and livestock-related conflict in northern and northwestern pastoral areas</t>
+  </si>
+  <si>
+    <t>2024-07</t>
+  </si>
+  <si>
+    <t>Nationwide anti-Finance Bill protests resulting in fatalities, destruction of property and temporary disruption of markets and transport</t>
+  </si>
+  <si>
+    <t>civil unrest</t>
+  </si>
+  <si>
+    <t>2026-07</t>
+  </si>
+  <si>
+    <t>Persistent localized intercommunal conflict and livestock rustling in pastoral counties affecting livelihoods and mobility</t>
+  </si>
+  <si>
+    <t>Widespread Desert Locust resurgence affecting vegetation and crops in northern Kenya</t>
+  </si>
+  <si>
+    <t>desert locust</t>
+  </si>
+  <si>
+    <t>agriculture</t>
+  </si>
+  <si>
+    <t>Regional Fall Armyworm not yet established in Kenya; no major national crop pest event reported</t>
+  </si>
+  <si>
+    <t>information</t>
+  </si>
+  <si>
+    <t>Recurring Quelea bird outbreaks causing localized cereal crop damage in eastern and coastal regions</t>
+  </si>
+  <si>
+    <t>quelea birds</t>
+  </si>
+  <si>
+    <t>Significant Quelea bird infestations affecting sorghum and rice production in several counties</t>
+  </si>
+  <si>
+    <t>Increased outbreaks of Maize Lethal Necrosis Disease (MLND) affecting maize-growing areas in the Rift Valley and western Kenya</t>
+  </si>
+  <si>
+    <t>crop disease</t>
+  </si>
+  <si>
+    <t>Continued spread of Maize Lethal Necrosis Disease reducing maize production in affected counties</t>
+  </si>
+  <si>
+    <t>First major national outbreak of Fall Armyworm causing widespread maize damage across the country</t>
+  </si>
+  <si>
+    <t>fall armyworm</t>
+  </si>
+  <si>
+    <t>Continued Fall Armyworm infestations requiring large-scale surveillance and control programmes</t>
+  </si>
+  <si>
+    <t>Desert Locust invasion affecting northern, eastern and central Kenya with extensive crop and pasture damage</t>
+  </si>
+  <si>
+    <t>Second generation Desert Locust swarms causing widespread damage despite ongoing control operations</t>
+  </si>
+  <si>
+    <t>Continued Desert Locust surveillance and localized swarm control with declining infestation levels</t>
+  </si>
+  <si>
+    <t>Continued Fall Armyworm infestations affecting maize production during successive cropping seasons</t>
+  </si>
+  <si>
+    <t>Recurring Quelea bird outbreaks affecting cereal production in irrigated and rainfed production zones</t>
+  </si>
+  <si>
+    <t>Continued endemic Fall Armyworm pressure requiring routine integrated pest management across maize-producing counties</t>
+  </si>
+  <si>
+    <t>No major nationwide crop pest outbreak; routine surveillance for Desert Locust, Fall Armyworm and MLND maintained</t>
+  </si>
+  <si>
+    <t>surveillance</t>
+  </si>
+  <si>
+    <t>2004-07</t>
+  </si>
+  <si>
+    <t>2005-03</t>
+  </si>
+  <si>
+    <t>2005-09</t>
+  </si>
+  <si>
+    <t>2006-04</t>
+  </si>
+  <si>
+    <t>2009-06</t>
+  </si>
+  <si>
+    <t>2010-05</t>
+  </si>
+  <si>
+    <t>2011-08</t>
+  </si>
+  <si>
+    <t>2012-04</t>
+  </si>
+  <si>
+    <t>2013-08</t>
+  </si>
+  <si>
+    <t>2016-08</t>
+  </si>
+  <si>
+    <t>2018-04</t>
+  </si>
+  <si>
+    <t>2019-05</t>
+  </si>
+  <si>
+    <t>enso_transition</t>
+  </si>
+  <si>
+    <t>Severe drought with widespread crop and livestock losses</t>
+  </si>
+  <si>
+    <t>Moderate El Niño with localized flooding</t>
+  </si>
+  <si>
+    <t>Multi-season drought across ASAL areas</t>
+  </si>
+  <si>
+    <t>El Niño enhanced short rains and flooding</t>
+  </si>
+  <si>
+    <t>La Niña-induced drought conditions</t>
+  </si>
+  <si>
+    <t>Strong La Niña with consecutive poor seasons</t>
+  </si>
+  <si>
+    <t>Consecutive below-average rainy seasons</t>
+  </si>
+  <si>
+    <t>Below-average rainfall in ASAL counties</t>
+  </si>
+  <si>
+    <t>Strong El Niño with widespread flooding</t>
+  </si>
+  <si>
+    <t>Consecutive failed rains causing severe drought</t>
+  </si>
+  <si>
+    <t>National drought emergency</t>
+  </si>
+  <si>
+    <t>Heavy long rains causing severe floods</t>
+  </si>
+  <si>
+    <t>Weak El Niño with above-average short rains</t>
+  </si>
+  <si>
+    <t>Widespread flooding along major rivers</t>
+  </si>
+  <si>
+    <t>Triple-dip La Niña intensifying drought</t>
+  </si>
+  <si>
+    <t>Record long rains and severe flooding</t>
+  </si>
+  <si>
+    <t>Recovery following favourable long rains</t>
+  </si>
+  <si>
+    <t>Weak La Niña with below-average short rains</t>
+  </si>
+  <si>
+    <t>Favourable long rains supporting recovery</t>
+  </si>
+  <si>
+    <t>Weak El Niño with enhanced short rains</t>
+  </si>
+  <si>
+    <t>Weak to moderate La Niña</t>
+  </si>
+  <si>
+    <t>Moderate to strong El Niño</t>
+  </si>
+  <si>
+    <t>Weak La Niña with continued rainfall deficits</t>
+  </si>
+  <si>
+    <t>Weak La Niña affecting rainfall distribution</t>
+  </si>
+  <si>
+    <t>Weak La Niña and poor short rains</t>
+  </si>
+  <si>
+    <t>Weak La Niña before wet long rains</t>
+  </si>
+  <si>
+    <t>Weak El Niño with wet short rains</t>
+  </si>
+  <si>
+    <t>Transition to ENSO-neutral conditions</t>
+  </si>
+  <si>
+    <t>Prolonged drought and food price increases</t>
+  </si>
+  <si>
+    <t>Multi-season drought and rising maize prices</t>
+  </si>
+  <si>
+    <t>Post-election violence disrupted markets</t>
+  </si>
+  <si>
+    <t>High inflation and maize shortages</t>
+  </si>
+  <si>
+    <t>Global food price spike and drought</t>
+  </si>
+  <si>
+    <t>El Niño market disruptions</t>
+  </si>
+  <si>
+    <t>Severe drought and maize price surge</t>
+  </si>
+  <si>
+    <t>Maize flour subsidy programme</t>
+  </si>
+  <si>
+    <t>Market recovery after drought</t>
+  </si>
+  <si>
+    <t>COVID-19 market disruptions</t>
+  </si>
+  <si>
+    <t>Prolonged drought and food inflation</t>
+  </si>
+  <si>
+    <t>Ukraine war and global price shock</t>
+  </si>
+  <si>
+    <t>Maize import waiver and subsidy</t>
+  </si>
+  <si>
+    <t>Fertilizer subsidy programme</t>
+  </si>
+  <si>
+    <t>Fuel price shock and weaker Shilling</t>
+  </si>
+  <si>
+    <t>Kenya Shilling depreciation</t>
+  </si>
+  <si>
+    <t>El Niño floods disrupted markets</t>
+  </si>
+  <si>
+    <t>Market stabilization and recovery</t>
+  </si>
+  <si>
+    <t>Middle East fuel price shock</t>
+  </si>
+  <si>
+    <t>drought, La Niña</t>
   </si>
 </sst>
 </file>
@@ -866,7 +1355,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -889,11 +1378,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -904,6 +1406,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1206,11 +1712,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F133"/>
+  <dimension ref="A1:F220"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" customWidth="1"/>
+    <col min="3" max="3" width="11.85546875" customWidth="1"/>
     <col min="4" max="4" width="78.85546875" customWidth="1"/>
     <col min="5" max="5" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
@@ -1237,22 +1744,22 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="7" t="s">
         <v>192</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="7" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2617,22 +3124,22 @@
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A71" s="1" t="s">
+      <c r="A71" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="B71" s="1" t="s">
+      <c r="B71" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="C71" s="1" t="s">
+      <c r="C71" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="D71" s="1" t="s">
+      <c r="D71" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="E71" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F71" s="1" t="s">
+      <c r="E71" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F71" s="7" t="s">
         <v>15</v>
       </c>
     </row>
@@ -3876,7 +4383,1746 @@
         <v>243</v>
       </c>
     </row>
+    <row r="134" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A134" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B134" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="C134" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="D134" s="6" t="s">
+        <v>310</v>
+      </c>
+      <c r="E134" s="6" t="s">
+        <v>311</v>
+      </c>
+      <c r="F134" s="6" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A135" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B135" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C135" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D135" s="6" t="s">
+        <v>312</v>
+      </c>
+      <c r="E135" s="6" t="s">
+        <v>311</v>
+      </c>
+      <c r="F135" s="6" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A136" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B136" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C136" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="D136" s="6" t="s">
+        <v>313</v>
+      </c>
+      <c r="E136" s="6" t="s">
+        <v>314</v>
+      </c>
+      <c r="F136" s="6" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A137" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B137" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C137" s="6" t="s">
+        <v>315</v>
+      </c>
+      <c r="D137" s="6" t="s">
+        <v>316</v>
+      </c>
+      <c r="E137" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="F137" s="6" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A138" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B138" s="6" t="s">
+        <v>288</v>
+      </c>
+      <c r="C138" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="D138" s="6" t="s">
+        <v>318</v>
+      </c>
+      <c r="E138" s="6" t="s">
+        <v>311</v>
+      </c>
+      <c r="F138" s="6" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A139" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B139" s="6" t="s">
+        <v>319</v>
+      </c>
+      <c r="C139" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="D139" s="6" t="s">
+        <v>320</v>
+      </c>
+      <c r="E139" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="F139" s="6" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A140" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B140" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="C140" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="D140" s="6" t="s">
+        <v>323</v>
+      </c>
+      <c r="E140" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="F140" s="6" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A141" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B141" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="C141" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="D141" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="E141" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="F141" s="6" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="142" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A142" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B142" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C142" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="D142" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="E142" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="F142" s="6" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="143" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A143" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B143" s="6" t="s">
+        <v>326</v>
+      </c>
+      <c r="C143" s="6" t="s">
+        <v>326</v>
+      </c>
+      <c r="D143" s="6" t="s">
+        <v>327</v>
+      </c>
+      <c r="E143" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="F143" s="6" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="144" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A144" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B144" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C144" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D144" s="6" t="s">
+        <v>328</v>
+      </c>
+      <c r="E144" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="F144" s="6" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="145" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A145" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B145" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C145" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D145" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="E145" s="6" t="s">
+        <v>311</v>
+      </c>
+      <c r="F145" s="6" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="146" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A146" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B146" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="C146" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="D146" s="6" t="s">
+        <v>331</v>
+      </c>
+      <c r="E146" s="6" t="s">
+        <v>314</v>
+      </c>
+      <c r="F146" s="6" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="147" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A147" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B147" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C147" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="D147" s="6" t="s">
+        <v>332</v>
+      </c>
+      <c r="E147" s="6" t="s">
+        <v>311</v>
+      </c>
+      <c r="F147" s="6" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A148" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B148" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C148" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="D148" s="6" t="s">
+        <v>333</v>
+      </c>
+      <c r="E148" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="F148" s="6" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="149" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A149" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B149" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="C149" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D149" s="6" t="s">
+        <v>334</v>
+      </c>
+      <c r="E149" s="6" t="s">
+        <v>311</v>
+      </c>
+      <c r="F149" s="6" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="150" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A150" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B150" s="6" t="s">
+        <v>335</v>
+      </c>
+      <c r="C150" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="D150" s="6" t="s">
+        <v>336</v>
+      </c>
+      <c r="E150" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="F150" s="6" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A151" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B151" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="C151" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="D151" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="E151" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F151" s="6" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="152" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A152" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B152" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C152" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D152" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="E152" s="6" t="s">
+        <v>311</v>
+      </c>
+      <c r="F152" s="6" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="153" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A153" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B153" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="C153" s="6" t="s">
+        <v>339</v>
+      </c>
+      <c r="D153" s="6" t="s">
+        <v>340</v>
+      </c>
+      <c r="E153" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="F153" s="6" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="154" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A154" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B154" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="C154" s="6" t="s">
+        <v>342</v>
+      </c>
+      <c r="D154" s="6" t="s">
+        <v>343</v>
+      </c>
+      <c r="E154" s="6" t="s">
+        <v>311</v>
+      </c>
+      <c r="F154" s="6" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="155" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A155" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B155" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C155" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="D155" s="6" t="s">
+        <v>344</v>
+      </c>
+      <c r="E155" s="6" t="s">
+        <v>345</v>
+      </c>
+      <c r="F155" s="6" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="156" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A156" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B156" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C156" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D156" s="6" t="s">
+        <v>347</v>
+      </c>
+      <c r="E156" s="6" t="s">
+        <v>348</v>
+      </c>
+      <c r="F156" s="6" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="157" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A157" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B157" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C157" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="D157" s="6" t="s">
+        <v>349</v>
+      </c>
+      <c r="E157" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="F157" s="6" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="158" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A158" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B158" s="6" t="s">
+        <v>319</v>
+      </c>
+      <c r="C158" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="D158" s="6" t="s">
+        <v>351</v>
+      </c>
+      <c r="E158" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="F158" s="6" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="159" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A159" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B159" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C159" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="D159" s="6" t="s">
+        <v>352</v>
+      </c>
+      <c r="E159" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="F159" s="6" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="160" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A160" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B160" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C160" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D160" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="E160" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="F160" s="6" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="161" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A161" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B161" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="C161" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D161" s="6" t="s">
+        <v>355</v>
+      </c>
+      <c r="E161" s="6" t="s">
+        <v>356</v>
+      </c>
+      <c r="F161" s="6" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="162" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A162" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B162" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C162" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="D162" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="E162" s="6" t="s">
+        <v>356</v>
+      </c>
+      <c r="F162" s="6" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="163" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A163" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B163" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="C163" s="6" t="s">
+        <v>303</v>
+      </c>
+      <c r="D163" s="6" t="s">
+        <v>358</v>
+      </c>
+      <c r="E163" s="6" t="s">
+        <v>345</v>
+      </c>
+      <c r="F163" s="6" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="164" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A164" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B164" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="C164" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D164" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="E164" s="6" t="s">
+        <v>345</v>
+      </c>
+      <c r="F164" s="6" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="165" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A165" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B165" s="6" t="s">
+        <v>335</v>
+      </c>
+      <c r="C165" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="D165" s="6" t="s">
+        <v>360</v>
+      </c>
+      <c r="E165" s="6" t="s">
+        <v>345</v>
+      </c>
+      <c r="F165" s="6" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="166" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A166" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B166" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="C166" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D166" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="E166" s="6" t="s">
+        <v>356</v>
+      </c>
+      <c r="F166" s="6" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="167" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A167" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B167" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C167" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D167" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="E167" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="F167" s="6" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="168" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A168" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B168" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="C168" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="D168" s="6" t="s">
+        <v>363</v>
+      </c>
+      <c r="E168" s="6" t="s">
+        <v>356</v>
+      </c>
+      <c r="F168" s="6" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="169" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A169" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B169" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="C169" s="6" t="s">
+        <v>342</v>
+      </c>
+      <c r="D169" s="6" t="s">
+        <v>364</v>
+      </c>
+      <c r="E169" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="F169" s="6" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="170" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A170" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B170" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="C170" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="D170" s="6" t="s">
+        <v>379</v>
+      </c>
+      <c r="E170" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="F170" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="171" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A171" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B171" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="C171" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="D171" s="6" t="s">
+        <v>380</v>
+      </c>
+      <c r="E171" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="F171" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="172" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A172" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B172" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="C172" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="D172" s="6" t="s">
+        <v>381</v>
+      </c>
+      <c r="E172" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="F172" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="173" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A173" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B173" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="C173" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D173" s="6" t="s">
+        <v>382</v>
+      </c>
+      <c r="E173" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="F173" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="174" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A174" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B174" s="6" t="s">
+        <v>285</v>
+      </c>
+      <c r="C174" s="6" t="s">
+        <v>286</v>
+      </c>
+      <c r="D174" s="6" t="s">
+        <v>383</v>
+      </c>
+      <c r="E174" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="F174" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="175" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A175" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B175" s="6" t="s">
+        <v>289</v>
+      </c>
+      <c r="C175" s="6" t="s">
+        <v>290</v>
+      </c>
+      <c r="D175" s="6" t="s">
+        <v>384</v>
+      </c>
+      <c r="E175" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="F175" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="176" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A176" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B176" s="6" t="s">
+        <v>291</v>
+      </c>
+      <c r="C176" s="6" t="s">
+        <v>292</v>
+      </c>
+      <c r="D176" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="E176" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="F176" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="177" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A177" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B177" s="6" t="s">
+        <v>293</v>
+      </c>
+      <c r="C177" s="6" t="s">
+        <v>294</v>
+      </c>
+      <c r="D177" s="6" t="s">
+        <v>386</v>
+      </c>
+      <c r="E177" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="F177" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="178" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A178" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B178" s="6" t="s">
+        <v>295</v>
+      </c>
+      <c r="C178" s="6" t="s">
+        <v>296</v>
+      </c>
+      <c r="D178" s="6" t="s">
+        <v>387</v>
+      </c>
+      <c r="E178" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="F178" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="179" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A179" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B179" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="C179" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="D179" s="6" t="s">
+        <v>388</v>
+      </c>
+      <c r="E179" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="F179" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="180" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A180" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B180" s="6" t="s">
+        <v>297</v>
+      </c>
+      <c r="C180" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="D180" s="6" t="s">
+        <v>389</v>
+      </c>
+      <c r="E180" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="F180" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="181" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A181" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B181" s="6" t="s">
+        <v>298</v>
+      </c>
+      <c r="C181" s="6" t="s">
+        <v>299</v>
+      </c>
+      <c r="D181" s="6" t="s">
+        <v>390</v>
+      </c>
+      <c r="E181" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="F181" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="182" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A182" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B182" s="6" t="s">
+        <v>300</v>
+      </c>
+      <c r="C182" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="D182" s="6" t="s">
+        <v>391</v>
+      </c>
+      <c r="E182" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="F182" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="183" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A183" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B183" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="C183" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="D183" s="6" t="s">
+        <v>392</v>
+      </c>
+      <c r="E183" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="F183" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="184" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A184" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B184" s="6" t="s">
+        <v>302</v>
+      </c>
+      <c r="C184" s="6" t="s">
+        <v>303</v>
+      </c>
+      <c r="D184" s="6" t="s">
+        <v>393</v>
+      </c>
+      <c r="E184" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="F184" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="185" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A185" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B185" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="C185" s="6" t="s">
+        <v>304</v>
+      </c>
+      <c r="D185" s="6" t="s">
+        <v>387</v>
+      </c>
+      <c r="E185" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="F185" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="186" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A186" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B186" s="6" t="s">
+        <v>305</v>
+      </c>
+      <c r="C186" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="D186" s="6" t="s">
+        <v>394</v>
+      </c>
+      <c r="E186" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="F186" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="187" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A187" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B187" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="C187" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="D187" s="6" t="s">
+        <v>395</v>
+      </c>
+      <c r="E187" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="F187" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="188" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A188" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B188" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C188" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="D188" s="6" t="s">
+        <v>396</v>
+      </c>
+      <c r="E188" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="F188" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="189" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A189" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B189" s="6" t="s">
+        <v>308</v>
+      </c>
+      <c r="C189" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D189" s="6" t="s">
+        <v>397</v>
+      </c>
+      <c r="E189" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="F189" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="190" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A190" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B190" s="6" t="s">
+        <v>366</v>
+      </c>
+      <c r="C190" s="6" t="s">
+        <v>367</v>
+      </c>
+      <c r="D190" s="6" t="s">
+        <v>398</v>
+      </c>
+      <c r="E190" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="F190" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="191" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A191" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B191" s="6" t="s">
+        <v>368</v>
+      </c>
+      <c r="C191" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="D191" s="6" t="s">
+        <v>399</v>
+      </c>
+      <c r="E191" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="F191" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="192" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A192" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B192" s="6" t="s">
+        <v>370</v>
+      </c>
+      <c r="C192" s="6" t="s">
+        <v>371</v>
+      </c>
+      <c r="D192" s="6" t="s">
+        <v>400</v>
+      </c>
+      <c r="E192" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="F192" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="193" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A193" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B193" s="6" t="s">
+        <v>372</v>
+      </c>
+      <c r="C193" s="6" t="s">
+        <v>373</v>
+      </c>
+      <c r="D193" s="6" t="s">
+        <v>401</v>
+      </c>
+      <c r="E193" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="F193" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="194" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A194" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B194" s="6" t="s">
+        <v>374</v>
+      </c>
+      <c r="C194" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="D194" s="6" t="s">
+        <v>402</v>
+      </c>
+      <c r="E194" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="F194" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="195" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A195" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B195" s="6" t="s">
+        <v>375</v>
+      </c>
+      <c r="C195" s="6" t="s">
+        <v>297</v>
+      </c>
+      <c r="D195" s="6" t="s">
+        <v>403</v>
+      </c>
+      <c r="E195" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="F195" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="196" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A196" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B196" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="C196" s="6" t="s">
+        <v>376</v>
+      </c>
+      <c r="D196" s="6" t="s">
+        <v>404</v>
+      </c>
+      <c r="E196" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="F196" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="197" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A197" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B197" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="C197" s="6" t="s">
+        <v>377</v>
+      </c>
+      <c r="D197" s="6" t="s">
+        <v>405</v>
+      </c>
+      <c r="E197" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="F197" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="198" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A198" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B198" s="6" t="s">
+        <v>339</v>
+      </c>
+      <c r="C198" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="D198" s="6" t="s">
+        <v>406</v>
+      </c>
+      <c r="E198" s="6" t="s">
+        <v>378</v>
+      </c>
+      <c r="F198" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="199" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A199" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B199" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="C199" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D199" s="6" t="s">
+        <v>407</v>
+      </c>
+      <c r="E199" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="F199" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="200" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A200" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B200" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C200" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D200" s="6" t="s">
+        <v>408</v>
+      </c>
+      <c r="E200" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F200" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="201" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A201" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B201" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C201" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="D201" s="6" t="s">
+        <v>409</v>
+      </c>
+      <c r="E201" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F201" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="202" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A202" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B202" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C202" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D202" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E202" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F202" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="203" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A203" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B203" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="C203" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="D203" s="6" t="s">
+        <v>410</v>
+      </c>
+      <c r="E203" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="F203" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="204" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A204" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B204" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C204" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D204" s="6" t="s">
+        <v>411</v>
+      </c>
+      <c r="E204" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="F204" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="205" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A205" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B205" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="C205" s="6" t="s">
+        <v>267</v>
+      </c>
+      <c r="D205" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E205" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="F205" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="206" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A206" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B206" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="C206" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="D206" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="E206" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="F206" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="207" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A207" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B207" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="C207" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="D207" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="E207" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="F207" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="208" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A208" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B208" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="C208" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="D208" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="E208" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="F208" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="209" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A209" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B209" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C209" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D209" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="E209" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="F209" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="210" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A210" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B210" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C210" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="D210" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="E210" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F210" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="211" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A211" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B211" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C211" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D211" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="E211" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="F211" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="212" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A212" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B212" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="C212" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D212" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="E212" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F212" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="213" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A213" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B213" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C213" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D213" s="6" t="s">
+        <v>418</v>
+      </c>
+      <c r="E213" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="F213" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="214" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A214" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B214" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="C214" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="D214" s="6" t="s">
+        <v>419</v>
+      </c>
+      <c r="E214" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="F214" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="215" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A215" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B215" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="C215" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D215" s="6" t="s">
+        <v>420</v>
+      </c>
+      <c r="E215" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="F215" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="216" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A216" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B216" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C216" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D216" s="6" t="s">
+        <v>421</v>
+      </c>
+      <c r="E216" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F216" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="217" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A217" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B217" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C217" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D217" s="6" t="s">
+        <v>422</v>
+      </c>
+      <c r="E217" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="F217" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="218" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A218" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B218" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="C218" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="D218" s="6" t="s">
+        <v>423</v>
+      </c>
+      <c r="E218" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="F218" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="219" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A219" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B219" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="C219" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="D219" s="6" t="s">
+        <v>424</v>
+      </c>
+      <c r="E219" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F219" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="220" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A220" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B220" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="C220" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D220" s="6" t="s">
+        <v>425</v>
+      </c>
+      <c r="E220" s="1"/>
+      <c r="F220" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:F220" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>